<commit_message>
Train a Skill L1 UB Balance: Low Role + Standing cartwheel standards
Coach standards (12 reps / 10 reps); prescriptions follow the L1
Locomotion role/cartwheel rows (total reps, each direction).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level1_Train_A_Skill_UB_Balance.xlsx
+++ b/Train_A_Skill/Level1_Train_A_Skill_UB_Balance.xlsx
@@ -113,12 +113,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
+        <fgColor rgb="FFEAF6E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF6E1"/>
+        <fgColor rgb="FFFFE599"/>
       </patternFill>
     </fill>
   </fills>
@@ -163,16 +163,16 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -999,14 +999,14 @@
           <t>Low Role</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>12 reps</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>8–12 total reps (4–6 each direction)</t>
         </is>
       </c>
     </row>
@@ -1493,14 +1493,14 @@
           <t>Standing cartwheel</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>10 reps</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>6–10 total reps (3–5 each direction)</t>
         </is>
       </c>
     </row>
@@ -1714,22 +1714,22 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>TEST: 2 Arm Croc Bent Leg</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>20s each side</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>10–20s each side · 2 sets</t>
         </is>
@@ -1744,22 +1744,22 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>TEST: Frog</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>15–30s · 2 sets</t>
         </is>
@@ -1774,22 +1774,22 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>TEST: Pencil Headstand</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>15–30s · 2 sets</t>
         </is>
@@ -1804,22 +1804,22 @@
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>TEST: Chest to wall pencil handstand hold</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>

</xml_diff>

<commit_message>
Train a Skill L1 UB Balance: TEST standard for Chest to wall pencil handstand hold
1-minute hold (coach); prescription 20–60s · 2 sets, same as the L1
Upper Body Chest to Wall Handstand Hold test. No open rows left.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level1_Train_A_Skill_UB_Balance.xlsx
+++ b/Train_A_Skill/Level1_Train_A_Skill_UB_Balance.xlsx
@@ -89,7 +89,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -116,11 +116,6 @@
         <fgColor rgb="FFEAF6E1"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -134,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -173,12 +168,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1814,14 +1803,14 @@
           <t>TEST: Chest to wall pencil handstand hold</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>1-minute hold</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>20–60s · 2 sets</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Train a Skill L1: freestyle rules (Foundation + Skill Work lists)
Each phase block splits into FOUNDATION (0s, indirect help, pick 1) and
SKILL WORK (numbered, direct help, pick 2 / only 1 -> do it twice);
3-4 sets each; pass = standard on 2 Foundation + 2 Skill Work (or the
1 on a 1-item list). Exercises, standards and prescriptions unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level1_Train_A_Skill_UB_Balance.xlsx
+++ b/Train_A_Skill/Level1_Train_A_Skill_UB_Balance.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FF0C1C0C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="FF9C6500"/>
       <sz val="9"/>
     </font>
@@ -89,7 +95,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +110,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE8B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D0B5"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -147,27 +158,30 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -535,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -553,10 +567,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each block is one skill — train only the skill you are chasing. Skills have different numbers of phases (set by the grades on the skill ladder); a skill only appears on the phase tabs it has. Phase 1 = that skill's 0 exercises + its grade 1 exercises. Self-paced — stay on each exercise until the standard is earned; train inside the PRESCRIPTION range, the top of the range is the STANDARD. ◇ PICK 1 = choose one. Every cell is a per-set prescription.</t>
+          <t>FREESTYLE — train only the skill you are chasing. Each session: 2–3 exercises, 3–4 sets each — 1 FOUNDATION (0 · indirect help: builds what the skill needs) + 2 SKILL WORK (numbered · direct help: the skill itself). Only 1 Skill Work exercise on the list → do it twice. PASS THE PHASE: hit the standard on 2 different Foundation + 2 different Skill Work exercises (a list with only 1 exercise → that 1 is enough). Phase 1 = Foundation + grade 1 Skill Work. Train inside the PRESCRIPTION range; the top of the range is the STANDARD. Every cell is a per-set prescription.</t>
         </is>
       </c>
     </row>
@@ -581,222 +595,254 @@
     <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2 ARM CROC BENT LEG  ·  BENT ARM BALANCE  ·  PHASE 1 of 3  ·  2 sets</t>
+          <t>2 ARM CROC BENT LEG  ·  BENT ARM BALANCE  ·  PHASE 1 of 3  ·  3–4 sets each</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 1: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
           <t>○  1</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>QDR Pushups</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>10 reps</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>6–10 reps</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>○  1</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Head + foot on floor QDR hold</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>20s hold each side</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>10–20s each side</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="8" customHeight="1"/>
-    <row r="10" ht="18.75" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>FROG  ·  BENT ARM BALANCE  ·  PHASE 1 of 3  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="10" ht="8" customHeight="1"/>
+    <row r="11" ht="18.75" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>FROG  ·  BENT ARM BALANCE  ·  PHASE 1 of 3  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 1: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>○  1</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Tripod Hold</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>15–30s</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="8" customHeight="1"/>
-    <row r="14" ht="18.75" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 1 of 4  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="15" ht="8" customHeight="1"/>
+    <row r="16" ht="18.75" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 1 of 4  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 1: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>○  1</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Tripod hold</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>15–30s</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="8" customHeight="1"/>
-    <row r="18" ht="18.75" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 1 of 5  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="20" ht="8" customHeight="1"/>
+    <row r="21" ht="18.75" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 1 of 5  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 1: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>○  1</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Pike handstand holds</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>1 minute hold</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>30–60s</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>○  1</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Low lateral monkey hop</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>12 reps (6 each side)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>8–12 reps each  (4–6 each side)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="8" customHeight="1"/>
+    <row r="26" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="D21:F21"/>
+  <mergeCells count="21">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="D19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="D12:F12"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -809,7 +855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -827,10 +873,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each block is one skill — train only the skill you are chasing. Skills have different numbers of phases (set by the grades on the skill ladder); a skill only appears on the phase tabs it has. Phase 2 = that skill's 0 exercises + its grade 2 exercises. Self-paced — stay on each exercise until the standard is earned; train inside the PRESCRIPTION range, the top of the range is the STANDARD. ◇ PICK 1 = choose one. Every cell is a per-set prescription.</t>
+          <t>FREESTYLE — train only the skill you are chasing. Each session: 2–3 exercises, 3–4 sets each — 1 FOUNDATION (0 · indirect help: builds what the skill needs) + 2 SKILL WORK (numbered · direct help: the skill itself). Only 1 Skill Work exercise on the list → do it twice. PASS THE PHASE: hit the standard on 2 different Foundation + 2 different Skill Work exercises (a list with only 1 exercise → that 1 is enough). Phase 2 = Foundation + grade 2 Skill Work. Train inside the PRESCRIPTION range; the top of the range is the STANDARD. Every cell is a per-set prescription.</t>
         </is>
       </c>
     </row>
@@ -855,198 +901,230 @@
     <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2 ARM CROC BENT LEG  ·  BENT ARM BALANCE  ·  PHASE 2 of 3  ·  2 sets</t>
+          <t>2 ARM CROC BENT LEG  ·  BENT ARM BALANCE  ·  PHASE 2 of 3  ·  3–4 sets each</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 2: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
           <t>○  2</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Head on floor QDR</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>20s hold each side</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>10–20s each side</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="8" customHeight="1"/>
-    <row r="9" ht="18.75" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>FROG  ·  BENT ARM BALANCE  ·  PHASE 2 of 3  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="9" ht="8" customHeight="1"/>
+    <row r="10" ht="18.75" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>FROG  ·  BENT ARM BALANCE  ·  PHASE 2 of 3  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 2: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>○  2</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Assisted Alternate Leg Frog</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>15–30s</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="8" customHeight="1"/>
-    <row r="13" ht="18.75" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 2 of 4  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="14" ht="8" customHeight="1"/>
+    <row r="15" ht="18.75" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 2 of 4  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 2: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>○  2</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Tuck headstand</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>15–30s</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="8" customHeight="1"/>
-    <row r="17" ht="18.75" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 2 of 5  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="19" ht="8" customHeight="1"/>
+    <row r="20" ht="18.75" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 2 of 5  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 2: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>○  2</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Low Role</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>12 reps</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>8–12 total reps (4–6 each direction)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>○  2</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Feet elevated handstand holds</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>1-minute hold on a 12–24 inch elevation</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>30–60s</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="8" customHeight="1"/>
+    <row r="25" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="20">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D24:F24"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A9:F9"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1059,7 +1137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1077,10 +1155,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each block is one skill — train only the skill you are chasing. Skills have different numbers of phases (set by the grades on the skill ladder); a skill only appears on the phase tabs it has. Phase 3 = that skill's 0 exercises + its grade 3 exercises. Self-paced — stay on each exercise until the standard is earned; train inside the PRESCRIPTION range, the top of the range is the STANDARD. ◇ PICK 1 = choose one. Every cell is a per-set prescription.</t>
+          <t>FREESTYLE — train only the skill you are chasing. Each session: 2–3 exercises, 3–4 sets each — 1 FOUNDATION (0 · indirect help: builds what the skill needs) + 2 SKILL WORK (numbered · direct help: the skill itself). Only 1 Skill Work exercise on the list → do it twice. PASS THE PHASE: hit the standard on 2 different Foundation + 2 different Skill Work exercises (a list with only 1 exercise → that 1 is enough). Phase 3 = Foundation + grade 3 Skill Work. Train inside the PRESCRIPTION range; the top of the range is the STANDARD. Every cell is a per-set prescription.</t>
         </is>
       </c>
     </row>
@@ -1105,222 +1183,254 @@
     <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2 ARM CROC BENT LEG  ·  BENT ARM BALANCE  ·  PHASE 3 of 3  ·  2 sets</t>
+          <t>2 ARM CROC BENT LEG  ·  BENT ARM BALANCE  ·  PHASE 3 of 3  ·  3–4 sets each</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 3: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
           <t>○  3</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Baby Freeze</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>20s each side hold</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>10–20s each side</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>○  3</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Elevated Croc Bent Legs</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>20s each side</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>10–20s each side</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="8" customHeight="1"/>
-    <row r="10" ht="18.75" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>FROG  ·  BENT ARM BALANCE  ·  PHASE 3 of 3  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="10" ht="8" customHeight="1"/>
+    <row r="11" ht="18.75" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>FROG  ·  BENT ARM BALANCE  ·  PHASE 3 of 3  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 3: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>○  3</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Head assisted frog</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>15–30s</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="8" customHeight="1"/>
-    <row r="14" ht="18.75" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 3 of 4  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="15" ht="8" customHeight="1"/>
+    <row r="16" ht="18.75" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 3 of 4  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 3: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>○  3</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Straddle Headstand</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>15–30s</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="8" customHeight="1"/>
-    <row r="18" ht="18.75" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 3 of 5  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="20" ht="8" customHeight="1"/>
+    <row r="21" ht="18.75" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 3 of 5  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 3: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>○  3</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Feet elevated scissor handstand switches</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>1 minute hold on a 12–24 inch elevation, switching legs every 5 seconds</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>30–60s · 12–24 inch elevation · switch legs every 5s</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>○  3</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Tuck lateral monkey hop</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>perform 12 total reps.</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>8–12 total reps</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="8" customHeight="1"/>
+    <row r="26" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="D21:F21"/>
+  <mergeCells count="21">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="D19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="D12:F12"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1333,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1351,10 +1461,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each block is one skill — train only the skill you are chasing. Skills have different numbers of phases (set by the grades on the skill ladder); a skill only appears on the phase tabs it has. Phase 4 = that skill's 0 exercises + its grade 4 exercises. Self-paced — stay on each exercise until the standard is earned; train inside the PRESCRIPTION range, the top of the range is the STANDARD. ◇ PICK 1 = choose one. Every cell is a per-set prescription.</t>
+          <t>FREESTYLE — train only the skill you are chasing. Each session: 2–3 exercises, 3–4 sets each — 1 FOUNDATION (0 · indirect help: builds what the skill needs) + 2 SKILL WORK (numbered · direct help: the skill itself). Only 1 Skill Work exercise on the list → do it twice. PASS THE PHASE: hit the standard on 2 different Foundation + 2 different Skill Work exercises (a list with only 1 exercise → that 1 is enough). Phase 4 = Foundation + grade 4 Skill Work. Train inside the PRESCRIPTION range; the top of the range is the STANDARD. Every cell is a per-set prescription.</t>
         </is>
       </c>
     </row>
@@ -1379,140 +1489,156 @@
     <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 4 of 4  ·  2 sets</t>
+          <t>PENCIL HEADSTAND  ·  BENT ARM BALANCE  ·  PHASE 4 of 4  ·  3–4 sets each</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+          <t>◇  THIS SESSION: 1 Skill Work × 2 (only 1 on the list)   ·   PASS PHASE 4: hit the standard on 1 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  only 1 — do it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
           <t>○  4</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Tuck to straddle headstand</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>10 reps</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>6–10 reps</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="8" customHeight="1"/>
-    <row r="9" ht="18.75" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 4 of 5  ·  2 sets</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="9" ht="8" customHeight="1"/>
+    <row r="10" ht="18.75" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 4 of 5  ·  3–4 sets each</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 4: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>○  4</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Back to wall handstand kick ups</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>5 reps on each side</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>3–5 Reps</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>○  4</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>45 degree handstand hold</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>1-minute hold</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>30–60 Seconds</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>○  4</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Standing cartwheel</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>10 reps</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>6–10 total reps (3–5 each direction)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="8" customHeight="1"/>
+    <row r="16" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="D12:F12"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1525,7 +1651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1543,10 +1669,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each block is one skill — train only the skill you are chasing. Skills have different numbers of phases (set by the grades on the skill ladder); a skill only appears on the phase tabs it has. Phase 5 = that skill's 0 exercises + its grade 5 exercises. Self-paced — stay on each exercise until the standard is earned; train inside the PRESCRIPTION range, the top of the range is the STANDARD. ◇ PICK 1 = choose one. Every cell is a per-set prescription.</t>
+          <t>FREESTYLE — train only the skill you are chasing. Each session: 2–3 exercises, 3–4 sets each — 1 FOUNDATION (0 · indirect help: builds what the skill needs) + 2 SKILL WORK (numbered · direct help: the skill itself). Only 1 Skill Work exercise on the list → do it twice. PASS THE PHASE: hit the standard on 2 different Foundation + 2 different Skill Work exercises (a list with only 1 exercise → that 1 is enough). Phase 5 = Foundation + grade 5 Skill Work. Train inside the PRESCRIPTION range; the top of the range is the STANDARD. Every cell is a per-set prescription.</t>
         </is>
       </c>
     </row>
@@ -1571,75 +1697,83 @@
     <row r="5" ht="18.75" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 5 of 5  ·  2 sets</t>
+          <t>CHEST TO WALL PENCIL HANDSTAND HOLD  ·  STRAIGHT ARM BALANCE  ·  PHASE 5 of 5  ·  3–4 sets each</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>◇  PICK 1  —  interchangeable, choose one</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+          <t>◇  THIS SESSION: 2 Skill Work   ·   PASS PHASE 5: hit the standard on 2 Skill Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>SKILL WORK  ·  direct help — the skill's own progression  ·  PICK 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
           <t>○  5</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Chest to wall pelvic tilts</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>10 reps</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>6–10 Reps</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>○  5</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Chest to wall scapula elevations</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>10 reps</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>6–10 Reps</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="8" customHeight="1"/>
+    <row r="10" ht="8" customHeight="1"/>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D9:F9"/>
     <mergeCell ref="D8:F8"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1703,22 +1837,22 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>TEST: 2 Arm Croc Bent Leg</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>20s each side</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>10–20s each side · 2 sets</t>
         </is>
@@ -1733,22 +1867,22 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>TEST: Frog</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>15–30s · 2 sets</t>
         </is>
@@ -1763,22 +1897,22 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>TEST: Pencil Headstand</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>30s hold</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>15–30s · 2 sets</t>
         </is>
@@ -1793,22 +1927,22 @@
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>✦</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>TEST: Chest to wall pencil handstand hold</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>1-minute hold</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>20–60s · 2 sets</t>
         </is>

</xml_diff>